<commit_message>
working heuristic, math checked
</commit_message>
<xml_diff>
--- a/Heuristic/data/test/Starting_point.xlsx
+++ b/Heuristic/data/test/Starting_point.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5ECFEFA-5A04-49B7-80B0-FDD7D17FD2BA}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5EA542A-8BDF-4B26-9C3F-43EA3E322264}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -1273,7 +1273,7 @@
         <v>25</v>
       </c>
       <c r="B7" s="15">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="8"/>

</xml_diff>